<commit_message>
plot time take sheet
</commit_message>
<xml_diff>
--- a/data/seizure_stage.xlsx
+++ b/data/seizure_stage.xlsx
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1863" uniqueCount="1631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1894" uniqueCount="1657">
   <si>
     <t>Stage</t>
   </si>
@@ -4955,6 +4955,84 @@
   </si>
   <si>
     <t>58:41 - 59:09</t>
+  </si>
+  <si>
+    <t>2:09 - 2:17</t>
+  </si>
+  <si>
+    <t>25:18 - 25:28</t>
+  </si>
+  <si>
+    <t>28:13 - 28:39</t>
+  </si>
+  <si>
+    <t>31:40 - 31:42</t>
+  </si>
+  <si>
+    <t>33:04 - 33:23</t>
+  </si>
+  <si>
+    <t>34:36 - 34:38</t>
+  </si>
+  <si>
+    <t>36:21 - 36:24</t>
+  </si>
+  <si>
+    <t>37:59 - 38:35</t>
+  </si>
+  <si>
+    <t>38:56 - 38:58</t>
+  </si>
+  <si>
+    <t>41:59 - 42:02</t>
+  </si>
+  <si>
+    <t>42:30 - 42:32</t>
+  </si>
+  <si>
+    <t>43:15 - 44:19</t>
+  </si>
+  <si>
+    <t>45:02 - 45:15</t>
+  </si>
+  <si>
+    <t>47:47 - 47:52</t>
+  </si>
+  <si>
+    <t>48:17 - 48:19</t>
+  </si>
+  <si>
+    <t>48:33 - 48:35</t>
+  </si>
+  <si>
+    <t>49:26 - 49:33</t>
+  </si>
+  <si>
+    <t>50:23 - 50:25</t>
+  </si>
+  <si>
+    <t>50:36 - 50:42</t>
+  </si>
+  <si>
+    <t>51:01 - 51:09</t>
+  </si>
+  <si>
+    <t>52:51 - 53:58</t>
+  </si>
+  <si>
+    <t>57:07 - 57:14</t>
+  </si>
+  <si>
+    <t>57:52 - 57:56</t>
+  </si>
+  <si>
+    <t>58:35 - 58:39</t>
+  </si>
+  <si>
+    <t>58:50 - 59:39</t>
+  </si>
+  <si>
+    <t>1:00:30 - 1:00:35</t>
   </si>
 </sst>
 </file>
@@ -28873,6 +28951,9 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="14.67"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
@@ -28883,6 +28964,269 @@
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>1631</v>
+      </c>
+      <c r="C2" s="7">
+        <v>46024.0</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>1632</v>
+      </c>
+      <c r="C3" s="7">
+        <v>46056.0</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="s">
+        <v>1633</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="D4" s="1"/>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="s">
+        <v>1634</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="s">
+        <v>1635</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="s">
+        <v>1636</v>
+      </c>
+      <c r="C7" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="s">
+        <v>1637</v>
+      </c>
+      <c r="C8" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="s">
+        <v>1638</v>
+      </c>
+      <c r="C9" s="7">
+        <v>46058.0</v>
+      </c>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="s">
+        <v>1639</v>
+      </c>
+      <c r="C10" s="1">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="s">
+        <v>913</v>
+      </c>
+      <c r="C11" s="1">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="s">
+        <v>1640</v>
+      </c>
+      <c r="C12" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="s">
+        <v>1641</v>
+      </c>
+      <c r="C13" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="s">
+        <v>1642</v>
+      </c>
+      <c r="C14" s="7">
+        <v>46058.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="s">
+        <v>1643</v>
+      </c>
+      <c r="C15" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="s">
+        <v>791</v>
+      </c>
+      <c r="C16" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="s">
+        <v>1644</v>
+      </c>
+      <c r="C17" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="s">
+        <v>1645</v>
+      </c>
+      <c r="C18" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="s">
+        <v>1646</v>
+      </c>
+      <c r="C19" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="s">
+        <v>1618</v>
+      </c>
+      <c r="C20" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="s">
+        <v>1647</v>
+      </c>
+      <c r="C21" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="s">
+        <v>1648</v>
+      </c>
+      <c r="C22" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="s">
+        <v>1649</v>
+      </c>
+      <c r="C23" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C24" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C25" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="s">
+        <v>1651</v>
+      </c>
+      <c r="C26" s="7">
+        <v>46056.0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C27" s="1">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="s">
+        <v>1652</v>
+      </c>
+      <c r="C28" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="s">
+        <v>1653</v>
+      </c>
+      <c r="C29" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="s">
+        <v>1654</v>
+      </c>
+      <c r="C30" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="s">
+        <v>1655</v>
+      </c>
+      <c r="C31" s="7">
+        <v>46056.0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C32" s="1">
+        <v>2.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>